<commit_message>
Itemize production materials and system equipment in quotation
- 제작물: 자료집(혹은 리플릿)·시나리오 큐카드·현수막·배너·폼보드·마이크택·명패·명찰·사전 티타임 개별 항목화
- 시스템: 노트북·프린터 임차 및 접수 소모품 반영
- 업무분장표 동기화 (마마미디어 VAT 포함 18,190,000원 유지)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018WmVGxh2eujqtEGBBBdyNp
</commit_message>
<xml_diff>
--- a/2026_취약노동자원탁회의_결과보고회/코리아스픽스_견적서_노사발전재단.xlsx
+++ b/2026_취약노동자원탁회의_결과보고회/코리아스픽스_견적서_노사발전재단.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="B9" s="6" t="n"/>
       <c r="C9" s="7">
-        <f>G51</f>
+        <f>G59</f>
         <v/>
       </c>
       <c r="D9" s="7" t="n"/>
@@ -839,7 +839,7 @@
       <c r="E16" s="10" t="n"/>
       <c r="F16" s="10" t="n"/>
       <c r="G16" s="11">
-        <f>SUM(G17:G22)</f>
+        <f>SUM(G17:G24)</f>
         <v/>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>원탁 배치·설치·철수</t>
+          <t>원탁 배치·무대·스크린 설치·철수</t>
         </is>
       </c>
       <c r="C19" s="12" t="n">
@@ -941,7 +941,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>리허설·현장 음향 운영</t>
+          <t>리허설·현장 음향·조명 운영</t>
         </is>
       </c>
       <c r="C20" s="12" t="n">
@@ -996,24 +996,24 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>접수 기자재</t>
+          <t>노트북 임차</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>노트북·프린터 등 접수 장비</t>
+          <t>발표 송출용 1대·접수용 1대</t>
         </is>
       </c>
       <c r="C22" s="12" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>식</t>
+          <t>대</t>
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="4" t="n">
         <v>2</v>
@@ -1024,34 +1024,48 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>3. 디자인 및 제작물</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="n"/>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n"/>
-      <c r="E23" s="10" t="n"/>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="11">
-        <f>SUM(G24:G28)</f>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>프린터 임차</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>레이저 프린터(현장 출력·명찰 재출력)</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>대</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="12">
+        <f>C23*E23*F23</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>키비주얼 디자인</t>
+          <t>접수 동선 셋팅·소모품</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>2회 공통 디자인</t>
+          <t>접수대 비품·토너·용지·필기구·멀티탭 등</t>
         </is>
       </c>
       <c r="C24" s="12" t="n">
-        <v>606000</v>
+        <v>100000</v>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
@@ -1062,7 +1076,7 @@
         <v>1</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G24" s="12">
         <f>C24*E24*F24</f>
@@ -1070,48 +1084,34 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>홍보·연출 인쇄물</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>X배너·현수막·폼보드 등</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="n">
-        <v>364000</v>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>식</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G25" s="12">
-        <f>C25*E25*F25</f>
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>3. 제작물</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="11">
+        <f>SUM(G26:G37)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>행사 자료집(리플릿)</t>
+          <t>키비주얼 디자인</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>원고 취합·편집·인쇄(60부 내외)</t>
+          <t>2회 공통 디자인(제작물 전반 적용)</t>
         </is>
       </c>
       <c r="C26" s="12" t="n">
-        <v>600000</v>
+        <v>606000</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
@@ -1122,7 +1122,7 @@
         <v>1</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G26" s="12">
         <f>C26*E26*F26</f>
@@ -1132,16 +1132,16 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>사회자 시나리오·큐카드</t>
+          <t>행사 자료집(혹은 리플릿) 편집</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>진행 시나리오 작성·큐카드 제작</t>
+          <t>원고 취합·편집디자인</t>
         </is>
       </c>
       <c r="C27" s="12" t="n">
-        <v>200000</v>
+        <v>300000</v>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
@@ -1162,24 +1162,24 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>명패·명찰·마이크택</t>
+          <t>행사 자료집(혹은 리플릿) 인쇄</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>참석자·발제자용</t>
+          <t>60부 내외(참석자 50명+예비)</t>
         </is>
       </c>
       <c r="C28" s="12" t="n">
-        <v>150000</v>
+        <v>5000</v>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>식</t>
+          <t>부</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F28" s="4" t="n">
         <v>2</v>
@@ -1190,45 +1190,59 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>4. 사진 및 영상 제작</t>
-        </is>
-      </c>
-      <c r="B29" s="10" t="n"/>
-      <c r="C29" s="10" t="n"/>
-      <c r="D29" s="10" t="n"/>
-      <c r="E29" s="10" t="n"/>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="11">
-        <f>SUM(G30:G33)</f>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>사회자 시나리오·큐카드</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>진행 시나리오 작성·큐카드 제작</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>식</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="12">
+        <f>C29*E29*F29</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>원탁회의 현장스케치 영상</t>
+          <t>현수막</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>'26년 원탁회의 스케치(2회 공통 상영)</t>
+          <t>행사장 메인 현수막</t>
         </is>
       </c>
       <c r="C30" s="12" t="n">
-        <v>606000</v>
+        <v>160000</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>편</t>
+          <t>개</t>
         </is>
       </c>
       <c r="E30" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G30" s="12">
         <f>C30*E30*F30</f>
@@ -1238,24 +1252,24 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>결과보고회 영상 촬영</t>
+          <t>배너</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>행사별 스케치 영상 촬영</t>
+          <t>X배너(입구·접수대)</t>
         </is>
       </c>
       <c r="C31" s="12" t="n">
-        <v>606000</v>
+        <v>60000</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>인</t>
+          <t>개</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F31" s="4" t="n">
         <v>2</v>
@@ -1268,24 +1282,24 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>결과보고회 사진 촬영</t>
+          <t>폼보드</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>행사·단체사진</t>
+          <t>안내·포토존 폼보드</t>
         </is>
       </c>
       <c r="C32" s="12" t="n">
-        <v>485000</v>
+        <v>42000</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>인</t>
+          <t>개</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32" s="4" t="n">
         <v>2</v>
@@ -1298,24 +1312,24 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>결과보고회 스케치 영상 편집</t>
+          <t>마이크택</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>행사별 결과영상</t>
+          <t>무선·유선 마이크용</t>
         </is>
       </c>
       <c r="C33" s="12" t="n">
-        <v>849000</v>
+        <v>15000</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>편</t>
+          <t>개</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F33" s="4" t="n">
         <v>2</v>
@@ -1326,42 +1340,56 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>5. 행사 진행 및 운영</t>
-        </is>
-      </c>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="10" t="n"/>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
-      <c r="G34" s="11">
-        <f>SUM(G35:G37)</f>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>명패</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>발제자·내빈 테이블 명패</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>개</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" s="12">
+        <f>C34*E34*F34</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>현장 운영 보조</t>
+          <t>명찰</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>행사보조·마이크 전달</t>
+          <t>참석자·스태프 명찰(케이스·목걸이 포함)</t>
         </is>
       </c>
       <c r="C35" s="12" t="n">
-        <v>243000</v>
+        <v>2500</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>인</t>
+          <t>개</t>
         </is>
       </c>
       <c r="E35" s="4" t="n">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="F35" s="4" t="n">
         <v>2</v>
@@ -1374,24 +1402,24 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>등록·접수 안내 인력</t>
+          <t>참석자 다과·생수</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>참석자 등록·안내·수당서명 접수</t>
+          <t>각 50명 기준</t>
         </is>
       </c>
       <c r="C36" s="12" t="n">
-        <v>200000</v>
+        <v>12000</v>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>인</t>
+          <t>명</t>
         </is>
       </c>
       <c r="E36" s="4" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="F36" s="4" t="n">
         <v>2</v>
@@ -1404,24 +1432,24 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>참석자 다과·생수</t>
+          <t>사전 티타임 준비</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>사전 티타임 포함, 각 50명 기준</t>
+          <t>내빈·발제자 10명 내외 다과·차·세팅</t>
         </is>
       </c>
       <c r="C37" s="12" t="n">
-        <v>12000</v>
+        <v>150000</v>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>명</t>
+          <t>식</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="F37" s="4" t="n">
         <v>2</v>
@@ -1434,7 +1462,7 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>6. 참가자 모집 및 관리</t>
+          <t>4. 사진 및 영상 제작</t>
         </is>
       </c>
       <c r="B38" s="10" t="n"/>
@@ -1443,34 +1471,34 @@
       <c r="E38" s="10" t="n"/>
       <c r="F38" s="10" t="n"/>
       <c r="G38" s="11">
-        <f>SUM(G39:G41)</f>
+        <f>SUM(G39:G42)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>참가자 모집·홍보</t>
+          <t>원탁회의 현장스케치 영상</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>홍보방안 수립·모집 안내·선발</t>
+          <t>'26년 원탁회의 스케치(2회 공통 상영)</t>
         </is>
       </c>
       <c r="C39" s="12" t="n">
-        <v>600000</v>
+        <v>606000</v>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>식</t>
+          <t>편</t>
         </is>
       </c>
       <c r="E39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G39" s="12">
         <f>C39*E39*F39</f>
@@ -1480,20 +1508,20 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>참가자 관리</t>
+          <t>결과보고회 영상 촬영</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>DB 관리·사전 안내(문자·유선)·참석 확인</t>
+          <t>행사별 스케치 영상 촬영</t>
         </is>
       </c>
       <c r="C40" s="12" t="n">
-        <v>300000</v>
+        <v>606000</v>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>식</t>
+          <t>인</t>
         </is>
       </c>
       <c r="E40" s="4" t="n">
@@ -1510,20 +1538,20 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>수당지급 서류 취합·제출</t>
+          <t>결과보고회 사진 촬영</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>수당지급명세서 작성·재단 제출</t>
+          <t>행사·단체사진</t>
         </is>
       </c>
       <c r="C41" s="12" t="n">
-        <v>300000</v>
+        <v>485000</v>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>식</t>
+          <t>인</t>
         </is>
       </c>
       <c r="E41" s="4" t="n">
@@ -1538,75 +1566,75 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="9" t="inlineStr">
-        <is>
-          <t>7. 출장 및 운송</t>
-        </is>
-      </c>
-      <c r="B42" s="10" t="n"/>
-      <c r="C42" s="10" t="n"/>
-      <c r="D42" s="10" t="n"/>
-      <c r="E42" s="10" t="n"/>
-      <c r="F42" s="10" t="n"/>
-      <c r="G42" s="11">
-        <f>SUM(G43:G44)</f>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>결과보고회 스케치 영상 편집</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>행사별 결과영상</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="n">
+        <v>849000</v>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>편</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="12">
+        <f>C42*E42*F42</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>출장·운송·숙박(제작·기술 인력)</t>
-        </is>
-      </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>장비·제작물 운송, 2회 합산</t>
-        </is>
-      </c>
-      <c r="C43" s="12" t="n">
-        <v>1590000</v>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>식</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" s="12">
-        <f>C43*E43*F43</f>
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>5. 행사 진행 및 운영</t>
+        </is>
+      </c>
+      <c r="B43" s="10" t="n"/>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="10" t="n"/>
+      <c r="E43" s="10" t="n"/>
+      <c r="F43" s="10" t="n"/>
+      <c r="G43" s="11">
+        <f>SUM(G44:G45)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>출장비(운영 인력)</t>
+          <t>현장 운영 보조</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>부산·대전 교통·숙박, 2회 합산</t>
+          <t>행사보조·마이크 전달</t>
         </is>
       </c>
       <c r="C44" s="12" t="n">
-        <v>800000</v>
+        <v>243000</v>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>식</t>
+          <t>인</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G44" s="12">
         <f>C44*E44*F44</f>
@@ -1614,154 +1642,366 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>등록·접수 안내 인력</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>참석자 등록·안내·수당서명 접수</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>인</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" s="12">
+        <f>C45*E45*F45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="9" t="inlineStr">
+        <is>
+          <t>6. 참가자 모집 및 관리</t>
+        </is>
+      </c>
+      <c r="B46" s="10" t="n"/>
+      <c r="C46" s="10" t="n"/>
+      <c r="D46" s="10" t="n"/>
+      <c r="E46" s="10" t="n"/>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="11">
+        <f>SUM(G47:G49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>참가자 모집·홍보</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>홍보방안 수립·모집 안내·선발</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="n">
+        <v>600000</v>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>식</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" s="12">
+        <f>C47*E47*F47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>참가자 관리</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>DB 관리·사전 안내(문자·유선)·참석 확인</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="n">
+        <v>300000</v>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>식</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G48" s="12">
+        <f>C48*E48*F48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>수당지급 서류 취합·제출</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>수당지급명세서 작성·재단 제출</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="n">
+        <v>300000</v>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>식</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" s="12">
+        <f>C49*E49*F49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>7. 출장 및 운송</t>
+        </is>
+      </c>
+      <c r="B50" s="10" t="n"/>
+      <c r="C50" s="10" t="n"/>
+      <c r="D50" s="10" t="n"/>
+      <c r="E50" s="10" t="n"/>
+      <c r="F50" s="10" t="n"/>
+      <c r="G50" s="11">
+        <f>SUM(G51:G52)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>출장·운송·숙박(제작·기술 인력)</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>장비·제작물 운송, 2회 합산</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="n">
+        <v>1590000</v>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>식</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="12">
+        <f>C51*E51*F51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>출장비(운영 인력)</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>부산·대전 교통·숙박, 2회 합산</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="n">
+        <v>800000</v>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>식</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="12">
+        <f>C52*E52*F52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
         <is>
           <t>직접비 소계</t>
         </is>
       </c>
-      <c r="B45" s="4" t="n"/>
-      <c r="C45" s="4" t="n"/>
-      <c r="D45" s="4" t="n"/>
-      <c r="E45" s="4" t="n"/>
-      <c r="F45" s="4" t="n"/>
-      <c r="G45" s="14">
-        <f>G12+G16+G23+G29+G34+G38+G42</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+      <c r="B53" s="4" t="n"/>
+      <c r="C53" s="4" t="n"/>
+      <c r="D53" s="4" t="n"/>
+      <c r="E53" s="4" t="n"/>
+      <c r="F53" s="4" t="n"/>
+      <c r="G53" s="14">
+        <f>G12+G16+G25+G38+G43+G46+G50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>일반관리비 (직접비 × 5%)</t>
         </is>
       </c>
-      <c r="B46" s="4" t="n"/>
-      <c r="C46" s="4" t="n"/>
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="4" t="n"/>
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="12">
-        <f>ROUND(G45*5%,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="B54" s="4" t="n"/>
+      <c r="C54" s="4" t="n"/>
+      <c r="D54" s="4" t="n"/>
+      <c r="E54" s="4" t="n"/>
+      <c r="F54" s="4" t="n"/>
+      <c r="G54" s="12">
+        <f>ROUND(G53*5%,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>기업이윤 ((직접비+일반관리비) × 5%)</t>
         </is>
       </c>
-      <c r="B47" s="4" t="n"/>
-      <c r="C47" s="4" t="n"/>
-      <c r="D47" s="4" t="n"/>
-      <c r="E47" s="4" t="n"/>
-      <c r="F47" s="4" t="n"/>
-      <c r="G47" s="12">
-        <f>ROUND((G45+G46)*5%,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="B55" s="4" t="n"/>
+      <c r="C55" s="4" t="n"/>
+      <c r="D55" s="4" t="n"/>
+      <c r="E55" s="4" t="n"/>
+      <c r="F55" s="4" t="n"/>
+      <c r="G55" s="12">
+        <f>ROUND((G53+G54)*5%,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>단수조정 (공급가액 만원 미만 절사)</t>
         </is>
       </c>
-      <c r="B48" s="4" t="n"/>
-      <c r="C48" s="4" t="n"/>
-      <c r="D48" s="4" t="n"/>
-      <c r="E48" s="4" t="n"/>
-      <c r="F48" s="4" t="n"/>
-      <c r="G48" s="12">
-        <f>ROUNDDOWN(G45+G46+G47,-4)-(G45+G46+G47)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="B56" s="4" t="n"/>
+      <c r="C56" s="4" t="n"/>
+      <c r="D56" s="4" t="n"/>
+      <c r="E56" s="4" t="n"/>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="12">
+        <f>ROUNDDOWN(G53+G54+G55,-4)-(G53+G54+G55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
         <is>
           <t>공급가액</t>
         </is>
       </c>
-      <c r="B49" s="4" t="n"/>
-      <c r="C49" s="4" t="n"/>
-      <c r="D49" s="4" t="n"/>
-      <c r="E49" s="4" t="n"/>
-      <c r="F49" s="4" t="n"/>
-      <c r="G49" s="14">
-        <f>G45+G46+G47+G48</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="B57" s="4" t="n"/>
+      <c r="C57" s="4" t="n"/>
+      <c r="D57" s="4" t="n"/>
+      <c r="E57" s="4" t="n"/>
+      <c r="F57" s="4" t="n"/>
+      <c r="G57" s="14">
+        <f>G53+G54+G55+G56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>부가가치세 (공급가액 × 10%)</t>
         </is>
       </c>
-      <c r="B50" s="4" t="n"/>
-      <c r="C50" s="4" t="n"/>
-      <c r="D50" s="4" t="n"/>
-      <c r="E50" s="4" t="n"/>
-      <c r="F50" s="4" t="n"/>
-      <c r="G50" s="12">
-        <f>ROUND(G49*10%,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="15" t="inlineStr">
+      <c r="B58" s="4" t="n"/>
+      <c r="C58" s="4" t="n"/>
+      <c r="D58" s="4" t="n"/>
+      <c r="E58" s="4" t="n"/>
+      <c r="F58" s="4" t="n"/>
+      <c r="G58" s="12">
+        <f>ROUND(G57*10%,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="15" t="inlineStr">
         <is>
           <t>합계 (부가가치세 포함)</t>
         </is>
       </c>
-      <c r="B51" s="6" t="n"/>
-      <c r="C51" s="6" t="n"/>
-      <c r="D51" s="6" t="n"/>
-      <c r="E51" s="6" t="n"/>
-      <c r="F51" s="6" t="n"/>
-      <c r="G51" s="16">
-        <f>G49+G50</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="17" t="inlineStr">
+      <c r="B59" s="6" t="n"/>
+      <c r="C59" s="6" t="n"/>
+      <c r="D59" s="6" t="n"/>
+      <c r="E59" s="6" t="n"/>
+      <c r="F59" s="6" t="n"/>
+      <c r="G59" s="16">
+        <f>G57+G58</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
         <is>
           <t>※ 비고</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="18" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="18" t="inlineStr">
         <is>
           <t>1. 행사장 대관료는 부산·대전 각 예산액 기준이며, 장소 확정 후 실제 임차료로 정산합니다. (재단 직접 계약 시 해당 금액 제외)</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="18" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="18" t="inlineStr">
         <is>
           <t>2. 참가자 사례비(참석수당)는 재단 부담으로 본 견적에서 제외하며, 수당지급명세서 취합·제출 업무는 포함합니다.</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="18" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="18" t="inlineStr">
         <is>
           <t>3. 전문사회자, 식사, 온라인 생중계, 시설 기본장비 외 추가 장비 임차는 제외(필요 시 별도 협의)입니다.</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="18" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="18" t="inlineStr">
         <is>
           <t>4. 인쇄물·자료집 수량 및 규격은 착수회의 시 확정하며, 변동 시 협의 후 조정합니다.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="18" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="18" t="inlineStr">
         <is>
           <t>5. 행사 일정·장소 변경 등 재단 요청사항 발생 시 상호 협의하여 조정합니다.</t>
         </is>
@@ -1771,42 +2011,42 @@
   <mergeCells count="38">
     <mergeCell ref="F4:G4"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A54:F54"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B3:C3"/>
-    <mergeCell ref="A53:G53"/>
+    <mergeCell ref="A62:G62"/>
     <mergeCell ref="F6:G6"/>
     <mergeCell ref="A12:F12"/>
     <mergeCell ref="A50:F50"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A63:G63"/>
     <mergeCell ref="F7:G7"/>
+    <mergeCell ref="A57:F57"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="D6:E6"/>
-    <mergeCell ref="A47:F47"/>
-    <mergeCell ref="A42:F42"/>
-    <mergeCell ref="A58:G58"/>
     <mergeCell ref="F5:G5"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A57:G57"/>
+    <mergeCell ref="A64:G64"/>
+    <mergeCell ref="A53:F53"/>
     <mergeCell ref="C9:G9"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A43:F43"/>
     <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A61:G61"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="D7:E7"/>
-    <mergeCell ref="A54:G54"/>
+    <mergeCell ref="A58:F58"/>
     <mergeCell ref="D4:E4"/>
-    <mergeCell ref="A34:F34"/>
-    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A65:G65"/>
     <mergeCell ref="D3:E3"/>
+    <mergeCell ref="A59:F59"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A49:F49"/>
-    <mergeCell ref="A51:F51"/>
-    <mergeCell ref="A56:G56"/>
+    <mergeCell ref="A66:G66"/>
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="A45:F45"/>
-    <mergeCell ref="A55:G55"/>
     <mergeCell ref="D5:E5"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="B4:C4"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>